<commit_message>
feat: classify signals as clinical AE vs administrative artifact
Adds signal_category as a first-class column in scripts/05's output (curated
against all 284 tested PTs, not just the consensus set) instead of leaving the
clinical/artifact distinction only in prose. Uses it in scripts/07 to clean up
figures that were mixing real adverse events with FAERS coding artifacts with
no visual cue: F3 forest plot now shows two separated, labeled blocks instead
of one flat ROR-ranked list; F2 volcano gets a 3-color split (signal/clinical/
administrative); F5 heatmap is restricted to the 4 clinical AE signals, since
a sex/age breakdown of "Off label use" isn't a meaningful question. T2/T3
tables get a Signal category column, and T3 is now grouped by category.
</commit_message>
<xml_diff>
--- a/outputs/tables/tables.xlsx
+++ b/outputs/tables/tables.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="T1_demographics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="T2_top_pts_by_frequency" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="T3_top_signals_by_strength" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="T4_soc_distribution" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="T5_time_to_onset" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T1_demographics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T2_top_pts_by_frequency" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T3_top_signals_by_strength" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T4_soc_distribution" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T5_time_to_onset" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -959,20 +959,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -990,50 +991,55 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Signal category</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>a (n cases)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>ROR</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>ROR 95% CI lower</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>ROR 95% CI upper</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>PRR</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>IC025</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>EBGM</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>EB05</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Label-listed (Y/N)</t>
         </is>
@@ -1045,34 +1051,39 @@
           <t>Disease progression</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Administrative/case-context</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>86</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>44.123</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="E4" s="4" t="n">
         <v>34.776</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="F4" s="4" t="n">
         <v>55.983</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="G4" s="4" t="n">
         <v>35.208</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>4.868</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>3.197</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>34.725</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>28.974</v>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1084,34 +1095,39 @@
           <t>Off label use</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Administrative/case-context</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>2.559</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>1.967</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>3.328</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>2.311</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>1.194</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>0.5649999999999999</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="J5" s="4" t="n">
         <v>2.295</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>1.865</v>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1123,34 +1139,39 @@
           <t>Stomatitis</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>59.115</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>45.234</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>77.25700000000001</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="G6" s="4" t="n">
         <v>50.175</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>5.171</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>3.029</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>49.195</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>39.85</v>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1162,34 +1183,39 @@
           <t>No adverse event</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Administrative/case-context</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>10.231</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>7.434</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>14.079</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="G7" s="4" t="n">
         <v>9.298999999999999</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>3.08</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>1.746</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>9.178000000000001</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>7.065</v>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1201,34 +1227,39 @@
           <t>Death</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D8" s="4" t="n">
         <v>1.643</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>1.096</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>2.462</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="G8" s="4" t="n">
         <v>1.604</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>0.665</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>-0.236</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>1.575</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>1.118</v>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1240,34 +1271,39 @@
           <t>Nausea</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D9" s="4" t="n">
         <v>1.498</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E9" s="4" t="n">
         <v>0.984</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>2.282</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>1.471</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>0.542</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>-0.372</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="J9" s="4" t="n">
         <v>1.442</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="K9" s="4" t="n">
         <v>1.008</v>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1279,34 +1315,39 @@
           <t>Fatigue</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="D10" s="4" t="n">
         <v>1.01</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="E10" s="4" t="n">
         <v>0.622</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>1.641</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="G10" s="4" t="n">
         <v>1.009</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>0.013</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>-0.945</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="J10" s="4" t="n">
         <v>0.983</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="K10" s="4" t="n">
         <v>0.646</v>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1318,34 +1359,39 @@
           <t>Interstitial lung disease</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="D11" s="4" t="n">
         <v>15.2</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E11" s="4" t="n">
         <v>9.214</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>25.073</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>14.654</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>3.371</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>1.026</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>14.176</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>9.183999999999999</v>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1357,34 +1403,39 @@
           <t>Infusion related reaction</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="D12" s="4" t="n">
         <v>7.338</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>4.305</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>12.508</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>7.125</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>2.555</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>0.608</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>6.882</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>4.318</v>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1396,34 +1447,39 @@
           <t>Dry eye</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="D13" s="4" t="n">
         <v>7.627</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="E13" s="4" t="n">
         <v>4.388</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>13.256</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="G13" s="4" t="n">
         <v>7.42</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>2.582</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>0.548</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="J13" s="4" t="n">
         <v>7.148</v>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="K13" s="4" t="n">
         <v>4.4</v>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1435,34 +1491,39 @@
           <t>Weight decreased</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>2.346</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>1.35</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>4.077</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>2.304</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>1.136</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="I14" s="4" t="n">
         <v>-0.24</v>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="J14" s="4" t="n">
         <v>2.224</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="K14" s="4" t="n">
         <v>1.369</v>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1474,34 +1535,39 @@
           <t>Alopecia</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="D15" s="4" t="n">
         <v>3.283</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="E15" s="4" t="n">
         <v>1.803</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>5.977</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="G15" s="4" t="n">
         <v>3.223</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>1.555</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="I15" s="4" t="n">
         <v>-0.1</v>
       </c>
-      <c r="I15" s="4" t="n">
+      <c r="J15" s="4" t="n">
         <v>3.089</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="K15" s="4" t="n">
         <v>1.817</v>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1513,34 +1579,39 @@
           <t>Dyspnoea</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="D16" s="4" t="n">
         <v>0.917</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="E16" s="4" t="n">
         <v>0.49</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="F16" s="4" t="n">
         <v>1.718</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>0.919</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>-0.116</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>-1.326</v>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="J16" s="4" t="n">
         <v>0.878</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>0.502</v>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1552,34 +1623,39 @@
           <t>Cough</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="D17" s="4" t="n">
         <v>1.522</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="E17" s="4" t="n">
         <v>0.8129999999999999</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>2.851</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>1.51</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>0.5590000000000001</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="I17" s="4" t="n">
         <v>-0.8129999999999999</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="J17" s="4" t="n">
         <v>1.442</v>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="K17" s="4" t="n">
         <v>0.824</v>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1591,34 +1667,39 @@
           <t>Rash</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="D18" s="4" t="n">
         <v>0.994</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="E18" s="4" t="n">
         <v>0.531</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="F18" s="4" t="n">
         <v>1.862</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="G18" s="4" t="n">
         <v>0.994</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>-0.008</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="I18" s="4" t="n">
         <v>-1.24</v>
       </c>
-      <c r="I18" s="4" t="n">
+      <c r="J18" s="4" t="n">
         <v>0.95</v>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="K18" s="4" t="n">
         <v>0.543</v>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1626,7 +1707,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1638,27 +1719,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table 3. Consensus signals ranked by ROR, all four algorithms (N=416 cases, datopotamab deruxtecan Primary Suspect, FAERS 2025Q1-2026Q1)</t>
+          <t>Table 3. Consensus signals by category (Clinical AE, then Administrative/case-context), ranked by ROR within each (N=416 cases, datopotamab deruxtecan Primary Suspect, FAERS 2025Q1-2026Q1)</t>
         </is>
       </c>
     </row>
@@ -1670,55 +1752,60 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Signal category</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>a (n cases)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>ROR</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>ROR 95% CI lower</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>ROR 95% CI upper</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>PRR</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>chi2 (Yates)</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>IC</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>IC025</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>EBGM</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>EB05</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Strict signal (+EB05&gt;2)</t>
         </is>
@@ -1730,277 +1817,312 @@
           <t>Stomatitis</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>59.115</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="E4" s="4" t="n">
         <v>45.234</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="F4" s="4" t="n">
         <v>77.25700000000001</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="G4" s="4" t="n">
         <v>50.175</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>3010.178</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>5.171</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>3.029</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>49.195</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>39.85</v>
       </c>
-      <c r="L4" s="4" t="b">
+      <c r="M4" s="4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Disease progression</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>86</v>
+          <t>Interstitial lung disease</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>44.123</v>
+        <v>16</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>34.776</v>
+        <v>15.2</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>55.983</v>
+        <v>9.214</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>35.208</v>
+        <v>25.073</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>2818.256</v>
+        <v>14.654</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>4.868</v>
+        <v>189.984</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>3.197</v>
+        <v>3.371</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>34.725</v>
+        <v>1.026</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>28.974</v>
-      </c>
-      <c r="L5" s="4" t="b">
+        <v>14.176</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>9.183999999999999</v>
+      </c>
+      <c r="M5" s="4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Prescribed underdose</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>9</v>
+          <t>Dry eye</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>19.292</v>
+        <v>13</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>9.952</v>
+        <v>7.627</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>37.397</v>
+        <v>4.388</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>18.896</v>
+        <v>13.256</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>134.736</v>
+        <v>7.42</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3.28</v>
+        <v>66.09699999999999</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.277</v>
+        <v>2.582</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>17.821</v>
+        <v>0.548</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>9.856999999999999</v>
-      </c>
-      <c r="L6" s="4" t="b">
+        <v>7.148</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="M6" s="4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Interstitial lung disease</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>16</v>
+          <t>Infusion related reaction</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Clinical AE</t>
+        </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>15.2</v>
+        <v>14</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>9.214</v>
+        <v>7.338</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>25.073</v>
+        <v>4.305</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>14.654</v>
+        <v>12.508</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>189.984</v>
+        <v>7.125</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>3.371</v>
+        <v>67.926</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1.026</v>
+        <v>2.555</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>14.176</v>
+        <v>0.608</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>9.183999999999999</v>
-      </c>
-      <c r="L7" s="4" t="b">
+        <v>6.882</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>4.318</v>
+      </c>
+      <c r="M7" s="4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>No adverse event</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>42</v>
+          <t>Disease progression</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Administrative/case-context</t>
+        </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>10.231</v>
+        <v>86</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>7.434</v>
+        <v>44.123</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>14.079</v>
+        <v>34.776</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>9.298999999999999</v>
+        <v>55.983</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>305.498</v>
+        <v>35.208</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3.08</v>
+        <v>2818.256</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1.746</v>
+        <v>4.868</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>9.178000000000001</v>
+        <v>3.197</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7.065</v>
-      </c>
-      <c r="L8" s="4" t="b">
+        <v>34.725</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>28.974</v>
+      </c>
+      <c r="M8" s="4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Dry eye</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>13</v>
+          <t>Prescribed underdose</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Administrative/case-context</t>
+        </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>7.627</v>
+        <v>9</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>4.388</v>
+        <v>19.292</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>13.256</v>
+        <v>9.952</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>7.42</v>
+        <v>37.397</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>66.09699999999999</v>
+        <v>18.896</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>2.582</v>
+        <v>134.736</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.548</v>
+        <v>3.28</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>7.148</v>
+        <v>0.277</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="L9" s="4" t="b">
+        <v>17.821</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>9.856999999999999</v>
+      </c>
+      <c r="M9" s="4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Infusion related reaction</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>14</v>
+          <t>No adverse event</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Administrative/case-context</t>
+        </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>7.338</v>
+        <v>42</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>4.305</v>
+        <v>10.231</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>12.508</v>
+        <v>7.434</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7.125</v>
+        <v>14.079</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>67.926</v>
+        <v>9.298999999999999</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>2.555</v>
+        <v>305.498</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>0.608</v>
+        <v>3.08</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6.882</v>
+        <v>1.746</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4.318</v>
-      </c>
-      <c r="L10" s="4" t="b">
+        <v>9.178000000000001</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>7.065</v>
+      </c>
+      <c r="M10" s="4" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2010,43 +2132,48 @@
           <t>Off label use</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Administrative/case-context</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="D11" s="4" t="n">
         <v>2.559</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E11" s="4" t="n">
         <v>1.967</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>3.328</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>2.311</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>51.292</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>1.194</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>0.5649999999999999</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>2.295</v>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>1.865</v>
       </c>
-      <c r="L11" s="4" t="b">
+      <c r="M11" s="4" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revise FAERS comparator hierarchy and signal rule
</commit_message>
<xml_diff>
--- a/outputs/tables/tables.xlsx
+++ b/outputs/tables/tables.xlsx
@@ -959,7 +959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -970,10 +970,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1016,30 +1013,15 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>PRR</t>
+          <t>IC</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>IC</t>
+          <t>IC025</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>IC025</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>EBGM</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>EB05</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Label-listed (Y/N)</t>
         </is>
@@ -1069,21 +1051,12 @@
         <v>55.983</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>35.208</v>
+        <v>4.868</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>4.868</v>
-      </c>
-      <c r="I4" s="4" t="n">
         <v>3.197</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>34.725</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>28.974</v>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1113,21 +1086,12 @@
         <v>3.328</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>2.311</v>
+        <v>1.194</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1.194</v>
-      </c>
-      <c r="I5" s="4" t="n">
         <v>0.5649999999999999</v>
       </c>
-      <c r="J5" s="4" t="n">
-        <v>2.295</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>1.865</v>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1157,21 +1121,12 @@
         <v>77.25700000000001</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>50.175</v>
+        <v>5.171</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>5.171</v>
-      </c>
-      <c r="I6" s="4" t="n">
         <v>3.029</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>49.195</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>39.85</v>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1201,21 +1156,12 @@
         <v>14.079</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>9.298999999999999</v>
+        <v>3.08</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="I7" s="4" t="n">
         <v>1.746</v>
       </c>
-      <c r="J7" s="4" t="n">
-        <v>9.178000000000001</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>7.065</v>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1245,21 +1191,12 @@
         <v>2.462</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>1.604</v>
+        <v>0.665</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.665</v>
-      </c>
-      <c r="I8" s="4" t="n">
         <v>-0.236</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>1.575</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>1.118</v>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1289,21 +1226,12 @@
         <v>2.282</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>1.471</v>
+        <v>0.542</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>0.542</v>
-      </c>
-      <c r="I9" s="4" t="n">
         <v>-0.372</v>
       </c>
-      <c r="J9" s="4" t="n">
-        <v>1.442</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>1.008</v>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1333,21 +1261,12 @@
         <v>1.641</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>1.009</v>
+        <v>0.013</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="I10" s="4" t="n">
         <v>-0.945</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>0.983</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>0.646</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1377,21 +1296,12 @@
         <v>25.073</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>14.654</v>
+        <v>3.371</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>3.371</v>
-      </c>
-      <c r="I11" s="4" t="n">
         <v>1.026</v>
       </c>
-      <c r="J11" s="4" t="n">
-        <v>14.176</v>
-      </c>
-      <c r="K11" s="4" t="n">
-        <v>9.183999999999999</v>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1421,21 +1331,12 @@
         <v>12.508</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>7.125</v>
+        <v>2.555</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>2.555</v>
-      </c>
-      <c r="I12" s="4" t="n">
         <v>0.608</v>
       </c>
-      <c r="J12" s="4" t="n">
-        <v>6.882</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>4.318</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1465,21 +1366,12 @@
         <v>13.256</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>7.42</v>
+        <v>2.582</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>2.582</v>
-      </c>
-      <c r="I13" s="4" t="n">
         <v>0.548</v>
       </c>
-      <c r="J13" s="4" t="n">
-        <v>7.148</v>
-      </c>
-      <c r="K13" s="4" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1509,21 +1401,12 @@
         <v>4.077</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>2.304</v>
+        <v>1.136</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>1.136</v>
-      </c>
-      <c r="I14" s="4" t="n">
         <v>-0.24</v>
       </c>
-      <c r="J14" s="4" t="n">
-        <v>2.224</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>1.369</v>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1553,21 +1436,12 @@
         <v>5.977</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>3.223</v>
+        <v>1.555</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>1.555</v>
-      </c>
-      <c r="I15" s="4" t="n">
         <v>-0.1</v>
       </c>
-      <c r="J15" s="4" t="n">
-        <v>3.089</v>
-      </c>
-      <c r="K15" s="4" t="n">
-        <v>1.817</v>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1597,21 +1471,12 @@
         <v>1.718</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.919</v>
+        <v>-0.116</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>-0.116</v>
-      </c>
-      <c r="I16" s="4" t="n">
         <v>-1.326</v>
       </c>
-      <c r="J16" s="4" t="n">
-        <v>0.878</v>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>0.502</v>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1641,21 +1506,12 @@
         <v>2.851</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>1.51</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.5590000000000001</v>
-      </c>
-      <c r="I17" s="4" t="n">
         <v>-0.8129999999999999</v>
       </c>
-      <c r="J17" s="4" t="n">
-        <v>1.442</v>
-      </c>
-      <c r="K17" s="4" t="n">
-        <v>0.824</v>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1685,21 +1541,12 @@
         <v>1.862</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.994</v>
+        <v>-0.008</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>-0.008</v>
-      </c>
-      <c r="I18" s="4" t="n">
         <v>-1.24</v>
       </c>
-      <c r="J18" s="4" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="K18" s="4" t="n">
-        <v>0.543</v>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1707,7 +1554,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1719,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -1728,19 +1575,14 @@
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table 3. Consensus signals by category (Clinical AE, then Administrative/case-context), ranked by ROR within each (N=416 cases, datopotamab deruxtecan Primary Suspect, FAERS 2025Q1-2026Q1)</t>
+          <t>Table 3. Primary ROR+IC signals by category (Clinical AE, then Administrative/case-context), ranked by ROR within each (N=416 cases, datopotamab deruxtecan Primary Suspect, FAERS 2025Q1-2026Q1)</t>
         </is>
       </c>
     </row>
@@ -1777,37 +1619,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>PRR</t>
+          <t>IC</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>chi2 (Yates)</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>IC</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
           <t>IC025</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>EBGM</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>EB05</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Strict signal (+EB05&gt;2)</t>
         </is>
       </c>
     </row>
@@ -1835,25 +1652,10 @@
         <v>77.25700000000001</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>50.175</v>
+        <v>5.171</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>3010.178</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>5.171</v>
-      </c>
-      <c r="J4" s="4" t="n">
         <v>3.029</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>49.195</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>39.85</v>
-      </c>
-      <c r="M4" s="4" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1880,25 +1682,10 @@
         <v>25.073</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>14.654</v>
+        <v>3.371</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>189.984</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>3.371</v>
-      </c>
-      <c r="J5" s="4" t="n">
         <v>1.026</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>14.176</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>9.183999999999999</v>
-      </c>
-      <c r="M5" s="4" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1925,25 +1712,10 @@
         <v>13.256</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>7.42</v>
+        <v>2.582</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>66.09699999999999</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>2.582</v>
-      </c>
-      <c r="J6" s="4" t="n">
         <v>0.548</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>7.148</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="M6" s="4" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1970,25 +1742,10 @@
         <v>12.508</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>7.125</v>
+        <v>2.555</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>67.926</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>2.555</v>
-      </c>
-      <c r="J7" s="4" t="n">
         <v>0.608</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>6.882</v>
-      </c>
-      <c r="L7" s="4" t="n">
-        <v>4.318</v>
-      </c>
-      <c r="M7" s="4" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -2015,25 +1772,10 @@
         <v>55.983</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>35.208</v>
+        <v>4.868</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2818.256</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>4.868</v>
-      </c>
-      <c r="J8" s="4" t="n">
         <v>3.197</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>34.725</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>28.974</v>
-      </c>
-      <c r="M8" s="4" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2060,25 +1802,10 @@
         <v>37.397</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>18.896</v>
+        <v>3.28</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>134.736</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="J9" s="4" t="n">
         <v>0.277</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>17.821</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>9.856999999999999</v>
-      </c>
-      <c r="M9" s="4" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -2105,25 +1832,10 @@
         <v>14.079</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>9.298999999999999</v>
+        <v>3.08</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>305.498</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>3.08</v>
-      </c>
-      <c r="J10" s="4" t="n">
         <v>1.746</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>9.178000000000001</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>7.065</v>
-      </c>
-      <c r="M10" s="4" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -2150,30 +1862,15 @@
         <v>3.328</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2.311</v>
+        <v>1.194</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>51.292</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>1.194</v>
-      </c>
-      <c r="J11" s="4" t="n">
         <v>0.5649999999999999</v>
-      </c>
-      <c r="K11" s="4" t="n">
-        <v>2.295</v>
-      </c>
-      <c r="L11" s="4" t="n">
-        <v>1.865</v>
-      </c>
-      <c r="M11" s="4" t="b">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>